<commit_message>
Add Match Day 23 section to Best 23 page
- Cascading filters: Round → Game for the selected season
- Loads actual match-day squads from match_ratings data
- Displays teams in Best 23 Comparison format with magnets
- Player name resolution via nickname variants (Cam→Cameron etc.)
- Falls back to match-level RatingPoints for unmatched players
- Reuses existing position grouping and conditional rating pills
- Data refresh (Round 5 match ratings, ladder, team stats)
</commit_message>
<xml_diff>
--- a/afl_ladders_2011_2026.xlsx
+++ b/afl_ladders_2011_2026.xlsx
@@ -14496,32 +14496,32 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Western Bulldogs</t>
+          <t>Sydney Swans</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="E271" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -14531,27 +14531,27 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>581</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>331</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>140.38%</t>
+          <t>175.53%</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>Won 4</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N271" t="n">
@@ -14566,19 +14566,19 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Sydney Swans</t>
+          <t>Fremantle Dockers</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="E272" t="inlineStr">
         <is>
           <t>1</t>
@@ -14591,37 +14591,37 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>481</t>
+          <t>444</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>338</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>182.89%</t>
+          <t>131.36%</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 4</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -14636,19 +14636,19 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Gold Coast Suns</t>
+          <t>Hawthorn Hawks</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>1</t>
@@ -14661,37 +14661,37 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>535</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>442</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>152.58%</t>
+          <t>121.04%</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 4</t>
         </is>
       </c>
       <c r="N273" t="n">
@@ -14706,19 +14706,19 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Fremantle Dockers</t>
+          <t>Western Bulldogs</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="E274" t="inlineStr">
         <is>
           <t>1</t>
@@ -14731,37 +14731,37 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>502</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>416</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>133.44%</t>
+          <t>120.67%</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>Won 3</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N274" t="n">
@@ -14776,12 +14776,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>North Melbourne Kangaroos</t>
+          <t>Gold Coast Suns</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -14791,7 +14791,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -14801,7 +14801,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -14811,27 +14811,27 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>541</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>410</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>115.32%</t>
+          <t>131.95%</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N275" t="n">
@@ -14846,12 +14846,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Hawthorn Hawks</t>
+          <t>Brisbane Lions</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -14861,7 +14861,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -14871,7 +14871,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -14881,22 +14881,22 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>490</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>426</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>114.02%</t>
+          <t>115.02%</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
@@ -14916,12 +14916,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Melbourne Demons</t>
+          <t>North Melbourne Kangaroos</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -14931,7 +14931,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -14941,7 +14941,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -14951,27 +14951,27 @@
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>450</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>425</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>102.05%</t>
+          <t>105.88%</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N277" t="n">
@@ -14986,24 +14986,24 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Port Adelaide Power</t>
+          <t>Geelong Cats</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="F278" t="inlineStr">
         <is>
           <t>0</t>
@@ -15011,32 +15011,32 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>460</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>453</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>117.65%</t>
+          <t>101.55%</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -15056,24 +15056,24 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Brisbane Lions</t>
+          <t>Melbourne Demons</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="F279" t="inlineStr">
         <is>
           <t>0</t>
@@ -15081,37 +15081,37 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>467</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>504</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>110.56%</t>
+          <t>92.66%</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>+0</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N279" t="n">
@@ -15126,7 +15126,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Adelaide Crows</t>
+          <t>Port Adelaide Power</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -15161,27 +15161,27 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>447</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>404</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>106.42%</t>
+          <t>110.64%</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N280" t="n">
@@ -15196,12 +15196,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Collingwood Magpies</t>
+          <t>Adelaide Crows</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
@@ -15231,27 +15231,27 @@
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>431</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>405</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>93.07%</t>
+          <t>106.42%</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N281" t="n">
@@ -15266,12 +15266,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Geelong Cats</t>
+          <t>GWS Giants</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -15281,7 +15281,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
@@ -15301,27 +15301,27 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>434</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>469</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>89.66%</t>
+          <t>92.54%</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N282" t="n">
@@ -15336,12 +15336,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>West Coast Eagles</t>
+          <t>Collingwood Magpies</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -15361,7 +15361,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
@@ -15371,27 +15371,27 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>348</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>377</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>64.85%</t>
+          <t>92.31%</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N283" t="n">
@@ -15411,12 +15411,12 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -15431,27 +15431,27 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>412</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>452</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>85.97%</t>
+          <t>91.15%</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
@@ -15461,7 +15461,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N284" t="n">
@@ -15476,17 +15476,17 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>GWS Giants</t>
+          <t>West Coast Eagles</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -15501,37 +15501,37 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>386</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>600</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>76.90%</t>
+          <t>64.33%</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Lost 3</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N285" t="n">
@@ -15621,47 +15621,47 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr">
+      <c r="F287" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr">
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>20.00%</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G287" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="H287" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>526</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>62.66%</t>
+          <t>76.05%</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Lost 4</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -15701,7 +15701,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -15721,17 +15721,17 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>297</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>527</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>56.06%</t>
+          <t>56.36%</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Lost 4</t>
+          <t>Lost 5</t>
         </is>
       </c>
       <c r="N288" t="n">

</xml_diff>

<commit_message>
Update AFL data, ladders, ratings and app for 2026 season
</commit_message>
<xml_diff>
--- a/afl_ladders_2011_2026.xlsx
+++ b/afl_ladders_2011_2026.xlsx
@@ -14501,12 +14501,12 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -14521,27 +14521,27 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>83.33%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>688</t>
+          <t>945</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>571</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>173.30%</t>
+          <t>165.50%</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>Won 3</t>
+          <t>Won 5</t>
         </is>
       </c>
       <c r="N271" t="n">
@@ -14571,12 +14571,12 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -14591,27 +14591,27 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>83.33%</t>
+          <t>87.50%</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>758</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>570</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>142.74%</t>
+          <t>132.98%</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -14621,7 +14621,7 @@
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Won 5</t>
+          <t>Won 7</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -14641,14 +14641,14 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>1</t>
@@ -14656,32 +14656,32 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>83.33%</t>
+          <t>81.25%</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>624</t>
+          <t>829</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>684</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>118.18%</t>
+          <t>121.20%</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>Won 5</t>
+          <t>Drew 1</t>
         </is>
       </c>
       <c r="N273" t="n">
@@ -14706,22 +14706,22 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Gold Coast Suns</t>
+          <t>Brisbane Lions</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -14731,27 +14731,27 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>62.50%</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>862</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>684</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>126.92%</t>
+          <t>126.02%</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -14761,7 +14761,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N274" t="n">
@@ -14776,22 +14776,22 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>North Melbourne Kangaroos</t>
+          <t>Gold Coast Suns</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -14801,27 +14801,27 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>62.50%</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>806</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>695</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>120.83%</t>
+          <t>115.97%</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
@@ -14851,17 +14851,17 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -14871,37 +14871,37 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>62.50%</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>591</t>
+          <t>791</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>690</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>116.11%</t>
+          <t>114.64%</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N276" t="n">
@@ -14916,22 +14916,22 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Western Bulldogs</t>
+          <t>Melbourne Demons</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -14941,27 +14941,27 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>62.50%</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>811</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>547</t>
+          <t>809</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>102.01%</t>
+          <t>100.25%</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
@@ -14971,7 +14971,7 @@
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 1</t>
         </is>
       </c>
       <c r="N277" t="n">
@@ -14986,12 +14986,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Melbourne Demons</t>
+          <t>Collingwood Magpies</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -15001,47 +15001,47 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>56.25%</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>666</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>606</t>
+          <t>613</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>94.22%</t>
+          <t>108.65%</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+0</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Won 1</t>
+          <t>Drew 1</t>
         </is>
       </c>
       <c r="N278" t="n">
@@ -15056,22 +15056,22 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Brisbane Lions</t>
+          <t>St Kilda Saints</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -15086,32 +15086,32 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>765</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>666</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>111.70%</t>
+          <t>114.86%</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Won 2</t>
         </is>
       </c>
       <c r="N279" t="n">
@@ -15126,22 +15126,22 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Adelaide Crows</t>
+          <t>North Melbourne Kangaroos</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -15156,32 +15156,32 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>764</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>507</t>
+          <t>720</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>105.33%</t>
+          <t>106.11%</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Won 2</t>
+          <t>Lost 2</t>
         </is>
       </c>
       <c r="N280" t="n">
@@ -15196,22 +15196,22 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Collingwood Magpies</t>
+          <t>Adelaide Crows</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -15226,22 +15226,22 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>685</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>709</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>94.78%</t>
+          <t>96.61%</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
@@ -15266,17 +15266,17 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Port Adelaide Power</t>
+          <t>Western Bulldogs</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -15291,27 +15291,27 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>720</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>493</t>
+          <t>787</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>108.11%</t>
+          <t>91.49%</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
@@ -15321,7 +15321,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Lost 2</t>
+          <t>Lost 4</t>
         </is>
       </c>
       <c r="N282" t="n">
@@ -15336,22 +15336,22 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>St Kilda Saints</t>
+          <t>Port Adelaide Power</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -15361,32 +15361,32 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>37.50%</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>514</t>
+          <t>703</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>634</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>92.61%</t>
+          <t>110.88%</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -15411,17 +15411,17 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -15431,32 +15431,32 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>37.50%</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>668</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>576</t>
+          <t>757</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>86.81%</t>
+          <t>88.24%</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>+0</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -15481,19 +15481,19 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="F285" t="inlineStr">
         <is>
           <t>0</t>
@@ -15501,7 +15501,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -15511,17 +15511,17 @@
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>557</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>697</t>
+          <t>939</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>61.26%</t>
+          <t>59.32%</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
@@ -15531,7 +15531,7 @@
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Lost 3</t>
+          <t>Lost 5</t>
         </is>
       </c>
       <c r="N285" t="n">
@@ -15551,7 +15551,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -15561,7 +15561,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -15571,7 +15571,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
@@ -15581,17 +15581,17 @@
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>634</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>601</t>
+          <t>812</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>79.20%</t>
+          <t>78.08%</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
@@ -15601,7 +15601,7 @@
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>Lost 4</t>
+          <t>Lost 6</t>
         </is>
       </c>
       <c r="N286" t="n">
@@ -15621,7 +15621,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -15631,7 +15631,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -15641,7 +15641,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -15651,17 +15651,17 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>649</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>925</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>79.07%</t>
+          <t>70.16%</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Lost 1</t>
+          <t>Lost 3</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -15691,47 +15691,47 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F288" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>523</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>657</t>
+          <t>871</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>53.58%</t>
+          <t>60.05%</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Lost 6</t>
+          <t>Won 1</t>
         </is>
       </c>
       <c r="N288" t="n">

</xml_diff>